<commit_message>
docs: add further verified QNLP papers
</commit_message>
<xml_diff>
--- a/metadata/QText.xlsx
+++ b/metadata/QText.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re93c57cfa63c4326"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R95bda723cb19466e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2313,50 +2313,336 @@
       </x:c>
       <x:c r="G70" s="3"/>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="3" t="str">
+        <x:v>Pretrained Quantum-Inspired Deep Neural Network for Natural Language Processing</x:v>
+      </x:c>
+      <x:c r="B71" s="3" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C71" s="3" t="str">
+        <x:v>IEEE</x:v>
+      </x:c>
+      <x:c r="D71" s="3" t="str">
+        <x:v>Jinjing Shi; Tian Chen; Wei Lai; Shichao Zhang; Xuelong Li</x:v>
+      </x:c>
+      <x:c r="E71" s="3" t="str">
+        <x:v>https://doi.org/10.1109/TCYB.2024.3398692</x:v>
+      </x:c>
+      <x:c r="F71" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G71" s="3"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="3" t="str">
+        <x:v>Comparing Natural Language Processing and Quantum Natural Processing approaches in text classification tasks</x:v>
+      </x:c>
+      <x:c r="B72" s="3" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C72" s="3" t="str">
+        <x:v>Elsevier</x:v>
+      </x:c>
+      <x:c r="D72" s="3" t="str">
+        <x:v>David Peral-García; Juan Cruz-Benito; Francisco José García-Peñalvo</x:v>
+      </x:c>
+      <x:c r="E72" s="3" t="str">
+        <x:v>https://doi.org/10.1016/j.eswa.2024.124427</x:v>
+      </x:c>
+      <x:c r="F72" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G72" s="3"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="3" t="str">
+        <x:v>These Aren’t the Vectors You’re Looking For: A Proof of Quantum Advantage in Compositional Generalization</x:v>
+      </x:c>
+      <x:c r="B73" s="3" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C73" s="3" t="str">
+        <x:v>Association for Computational Linguistics</x:v>
+      </x:c>
+      <x:c r="D73" s="3" t="str">
+        <x:v>Karthik Srikumar</x:v>
+      </x:c>
+      <x:c r="E73" s="3" t="str">
+        <x:v>https://aclanthology.org/2025.quantumnlp-1.2/</x:v>
+      </x:c>
+      <x:c r="F73" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G73" s="3"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="3" t="str">
+        <x:v>Hybrid Classical-Quantum Framework for Sentiment Classification and Claim Check-Worthiness Identification in Bengali</x:v>
+      </x:c>
+      <x:c r="B74" s="3" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C74" s="3" t="str">
+        <x:v>Association for Computational Linguistics</x:v>
+      </x:c>
+      <x:c r="D74" s="3" t="str">
+        <x:v>Pritam Pal; Dipankar Das; Anup Kumar Kolya; Siddhartha Bhattacharyya</x:v>
+      </x:c>
+      <x:c r="E74" s="3" t="str">
+        <x:v>https://aclanthology.org/2025.quantumnlp-1.3/</x:v>
+      </x:c>
+      <x:c r="F74" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G74" s="3"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="3" t="str">
+        <x:v>A Hybrid Quantum-Classical Fusion for Deep Semantic Paraphrase Detection</x:v>
+      </x:c>
+      <x:c r="B75" s="3" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C75" s="3" t="str">
+        <x:v>Association for Computational Linguistics</x:v>
+      </x:c>
+      <x:c r="D75" s="3" t="str">
+        <x:v>Devanarayanan K; Fayas S Mohamad; Dheeraj V Mohan; Reshma Sheik</x:v>
+      </x:c>
+      <x:c r="E75" s="3" t="str">
+        <x:v>https://aclanthology.org/2025.quantumnlp-1.4/</x:v>
+      </x:c>
+      <x:c r="F75" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G75" s="3"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="3" t="str">
+        <x:v>Quantum-Enhanced Gated Recurrent Units for Part-of-Speech Tagging</x:v>
+      </x:c>
+      <x:c r="B76" s="3" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C76" s="3" t="str">
+        <x:v>Association for Computational Linguistics</x:v>
+      </x:c>
+      <x:c r="D76" s="3" t="str">
+        <x:v>Ashutosh Rai; Shyambabu Pandey; Partha Pakray</x:v>
+      </x:c>
+      <x:c r="E76" s="3" t="str">
+        <x:v>https://aclanthology.org/2025.quantumnlp-1.5/</x:v>
+      </x:c>
+      <x:c r="F76" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G76" s="3"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="3" t="str">
+        <x:v>A Review of Quantum Computing Approaches to Semantic Search and Text Classification in Natural Language Processing</x:v>
+      </x:c>
+      <x:c r="B77" s="3" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C77" s="3" t="str">
+        <x:v>Association for Computational Linguistics</x:v>
+      </x:c>
+      <x:c r="D77" s="3" t="str">
+        <x:v>Sauvik Bal</x:v>
+      </x:c>
+      <x:c r="E77" s="3" t="str">
+        <x:v>https://aclanthology.org/2025.quantumnlp-1.6/</x:v>
+      </x:c>
+      <x:c r="F77" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G77" s="3"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="3" t="str">
+        <x:v>A Quantum Self-Attention Neural Network Model on Quantum Circuits</x:v>
+      </x:c>
+      <x:c r="B78" s="3" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C78" s="3" t="str">
+        <x:v>IEEE</x:v>
+      </x:c>
+      <x:c r="D78" s="3" t="str">
+        <x:v>Jin Zheng; Qing Gao; Daoyi Dong; Maciej Ogorzalek; Yi Du</x:v>
+      </x:c>
+      <x:c r="E78" s="3" t="str">
+        <x:v>https://doi.org/10.1109/TCYB.2026.3704405</x:v>
+      </x:c>
+      <x:c r="F78" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G78" s="3"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="3" t="str">
+        <x:v>Quantum Methods for Managing Ambiguity in Natural Language Processing</x:v>
+      </x:c>
+      <x:c r="B79" s="3" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C79" s="3" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D79" s="3" t="str">
+        <x:v>Jurek Eisinger; Ward Gauderis; Lin de Huybrecht; Geraint A. Wiggins</x:v>
+      </x:c>
+      <x:c r="E79" s="3" t="str">
+        <x:v>https://doi.org/10.1007/s42484-026-00421-5</x:v>
+      </x:c>
+      <x:c r="F79" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G79" s="3"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="3" t="str">
+        <x:v>Exploring all-quantum long short-term memory networks to enhance text sentiment classification</x:v>
+      </x:c>
+      <x:c r="B80" s="3" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C80" s="3" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D80" s="3" t="str">
+        <x:v>Feng Yan; Jun Yang; Kazuhiro Kawamoto; Kiyoshi Hirota</x:v>
+      </x:c>
+      <x:c r="E80" s="3" t="str">
+        <x:v>https://doi.org/10.1007/s11128-026-05236-8</x:v>
+      </x:c>
+      <x:c r="F80" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G80" s="3"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="3" t="str">
+        <x:v>QTopic: A novel quantum perspective on learning topics from text</x:v>
+      </x:c>
+      <x:c r="B81" s="3" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C81" s="3" t="str">
+        <x:v>Elsevier</x:v>
+      </x:c>
+      <x:c r="D81" s="3" t="str">
+        <x:v>Monika Kabir; Mohammed Kaosar; Ferdous Sohel</x:v>
+      </x:c>
+      <x:c r="E81" s="3" t="str">
+        <x:v>https://doi.org/10.1016/j.neucom.2025.132483</x:v>
+      </x:c>
+      <x:c r="F81" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G81" s="3"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="3" t="str">
+        <x:v>Unlocking the power of quantum computing in biomedical NLP for lung cancer diagnosis</x:v>
+      </x:c>
+      <x:c r="B82" s="3" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C82" s="3" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D82" s="3" t="str">
+        <x:v>Cyrille YetuYetu Kesiku; Begonya Garcia-Zapirain; Adel S. Elmaghraby</x:v>
+      </x:c>
+      <x:c r="E82" s="3" t="str">
+        <x:v>https://doi.org/10.1007/s42484-026-00392-7</x:v>
+      </x:c>
+      <x:c r="F82" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G82" s="3"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="3" t="str">
+        <x:v>Quantum-Inspired Transformers for Scalable Natural Language Processing Applications in Future AI</x:v>
+      </x:c>
+      <x:c r="B83" s="3" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C83" s="3" t="str">
+        <x:v>Elsevier</x:v>
+      </x:c>
+      <x:c r="D83" s="3" t="str">
+        <x:v>Priya Vij; Parmanand Yadav</x:v>
+      </x:c>
+      <x:c r="E83" s="3" t="str">
+        <x:v>https://doi.org/10.1016/j.procs.2026.01.020</x:v>
+      </x:c>
+      <x:c r="F83" s="3" t="str">
+        <x:v>Qtext</x:v>
+      </x:c>
+      <x:c r="G83" s="3"/>
+    </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="Rd5b7fffc62514173"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="Re756e637163f4650"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="R44d13ac1309a43c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="R8f5bff644ef84589"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="Rbab3f697139a4fa1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R5a92a6d27fe243b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="Ra9be5b7ccbb34123"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R78639396e71644ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R6473166473594601"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="R1ba2232cd9c24ab7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="R9ce1fa4abaf94097"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R46017a97c19a44a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R56695dfaa10448d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="R3db42abefb3844cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="R18d865dc43ff4d16"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Re8b8672c63344254"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R364ae9c3a2bd4471"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R60da3ac176804e99"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R521d8fd4c2c64359"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R250e2203b4df49fc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R7cb5054e3ff04d93"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="Rf13916a93da342ee"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Re6f154ed978148f0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R42dcfd9a60fa4216"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="Re31b8a66438448dc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="Rb8b13f5aa11447df"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="Rfc82fef62a74420c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R57029ec264bb4fba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Rc0113f8d0cc24f17"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R95c987af3c534a2f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R2fa18100ff4a48bd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R663a949cdb99443f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="Rf04a9550e5c84a22"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="Ref34146f6bea4faf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R8fdd37f3862c4359"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R86a354fdfd8648a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="Rf7ea4a47ab4e44e3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="R9f3f608ab4554bca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R2cb305303f73476a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Rb55b07e42e0e4579"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="Rd81ed7fcf3e041c9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R80e169efc1f34ded"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="Rf7c6c3f4b32f4f18"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="R80fb2c87ae744bf5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="Rc13cf020a0384b35"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="Rf6f1582d6e624fa9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="R50e24dd5b7c04649"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R267d9101b91e40fb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R6b9cbb7a55e948ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="Rda71d92417214eff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="R50cda409064d4c24"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="R70b5a129167d4ed7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="R70425aadf88b4eba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R585675e50a9a4e16"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="Rabd21113c70246db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="R2e6a2204107640cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="R7a233f704e7b4556"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Raeb217e1c38847b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="R52145b5d6dc64b97"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R2c13681d24f24918"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R803d6003bf634a40"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="R5ade6f69da2f4d82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R4a76fbe9dc394c14"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R78874b6e18f04050"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Rc284f7fbf1804b11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R21981071745b4cf7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R90f6a2bfa05f4a1a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R39cbd3822d85439e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R3b179c994505483d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R2b589c9f0a71460d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Rcf67fb0df6784c1a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R41b52c7d1e374cc6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="Rcf1b5c9732cb4046"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R28e764650bdd4e47"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R48f6f5885928490d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="R77c0366de45a4b3c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R1f9b27bda8144b47"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="Rc488c0bb8e0b42fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R06db5093af65468b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="R614cf216dba94c3e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R3b846d5d87664ae6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="R1deec6a1d2a84e58"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="R6b24b790f10544ff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="Rb2c1dbaa40304a25"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="R10f81fc5ed5f4d0a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R10320d06ba414515"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="R4a1274577cf74caf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="R252f2b4119ea44b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Rd44d01503c1644d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="Rd5bd541dcca94454"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R2f4d2fa0e08f4288"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="Ra45c06370f1a4392"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="Rd8c9a20b3a7f4e13"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="Rd2870aef55014225"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="Rc5519895eacd491e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="Rd333336e66ec4c35"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="Rabd7b27a6eaf4cce"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>